<commit_message>
Updated app to remove camera
</commit_message>
<xml_diff>
--- a/SqueezeReviews.xlsx
+++ b/SqueezeReviews.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rmazorow/Documents/Squeeze-Threshold-Verification/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B98BF45-0F5C-3B47-8F4B-09CE41111AC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9711BD43-F14E-9849-953C-ECC784B21D7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="94" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="29" uniqueCount="17">
   <si>
     <t>R02</t>
   </si>
@@ -46,6 +46,9 @@
     <t>SubID</t>
   </si>
   <si>
+    <t>WTest1</t>
+  </si>
+  <si>
     <t>Block</t>
   </si>
   <si>
@@ -73,12 +76,6 @@
     <t>FilePath</t>
   </si>
   <si>
-    <t>Camera</t>
-  </si>
-  <si>
-    <t>opti</t>
-  </si>
-  <si>
     <t>WTest1/S_01/_trial001_2026-04-14_13-26-41.mat</t>
   </si>
   <si>
@@ -92,39 +89,6 @@
   </si>
   <si>
     <t>WTest1/S_01/_trial005_2026-04-14_13-29-25.mat</t>
-  </si>
-  <si>
-    <t>WTest1</t>
-  </si>
-  <si>
-    <t>WTest2</t>
-  </si>
-  <si>
-    <t>WTest3</t>
-  </si>
-  <si>
-    <t>WTest4</t>
-  </si>
-  <si>
-    <t>WTest5</t>
-  </si>
-  <si>
-    <t>S_02</t>
-  </si>
-  <si>
-    <t>WTest1/S_02/_trial001_2026-04-28_16-31-08.mat</t>
-  </si>
-  <si>
-    <t>WTest1/S_02/_trial002_2026-04-28_16-31-27.mat</t>
-  </si>
-  <si>
-    <t>WTest1/S_02/_trial003_2026-04-28_16-31-47.mat</t>
-  </si>
-  <si>
-    <t>WTest1/S_02/_trial004_2026-04-28_16-32-10.mat</t>
-  </si>
-  <si>
-    <t>WTest1/S_02/_trial005_2026-04-28_16-32-32.mat</t>
   </si>
 </sst>
 </file>
@@ -512,7 +476,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C9FC292-298F-7347-9E2B-E19B83CAC426}">
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.7109375" customWidth="true"/>
@@ -522,45 +486,42 @@
     <col min="6" max="6" width="10.7109375" customWidth="true"/>
     <col min="7" max="7" width="9.7109375" customWidth="true"/>
     <col min="8" max="8" width="46.7109375" customWidth="true"/>
-    <col min="9" max="9" width="7.7109375" customWidth="true"/>
+    <col min="9" max="9" width="7.6640625" customWidth="true"/>
     <col min="3" max="3" width="6.7109375" customWidth="true"/>
   </cols>
   <sheetData>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.2">
+    <row r="1">
       <c r="A1" s="0" t="s">
         <v>1</v>
       </c>
       <c r="B1" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="H1" s="0" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="B2" s="0" t="s">
         <v>4</v>
-      </c>
-      <c r="D1" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="E1" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="F1" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="G1" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="H1" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="I1" s="0" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.2">
-      <c r="A2" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="B2" s="0" t="s">
-        <v>3</v>
       </c>
       <c r="C2" s="0">
         <v>1</v>
@@ -575,21 +536,18 @@
         <v>1896</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="I2" s="0" t="s">
         <v>12</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.2">
+    <row r="3">
       <c r="A3" s="0" t="s">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C3" s="0">
         <v>2</v>
@@ -604,21 +562,18 @@
         <v>2828</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="I3" s="0" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4">
       <c r="A4" s="0" t="s">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C4" s="0">
         <v>3</v>
@@ -633,21 +588,18 @@
         <v>3836</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="I4" s="0" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5">
       <c r="A5" s="0" t="s">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C5" s="0">
         <v>4</v>
@@ -662,21 +614,18 @@
         <v>1838</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>16</v>
-      </c>
-      <c r="I5" s="0" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.2">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6">
       <c r="A6" s="0" t="s">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C6" s="0">
         <v>5</v>
@@ -691,158 +640,10 @@
         <v>2031</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>17</v>
-      </c>
-      <c r="I6" s="0" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" s="0">
-        <v>1</v>
-      </c>
-      <c r="D7" s="0">
-        <v>1765</v>
-      </c>
-      <c r="E7" s="0">
-        <v>1817</v>
-      </c>
-      <c r="F7" s="0">
-        <v>2218</v>
-      </c>
-      <c r="G7" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="H7" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="I7" s="0" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="C8" s="0">
-        <v>2</v>
-      </c>
-      <c r="D8" s="0">
-        <v>1663</v>
-      </c>
-      <c r="E8" s="0">
-        <v>1711</v>
-      </c>
-      <c r="F8" s="0">
-        <v>2112</v>
-      </c>
-      <c r="G8" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="H8" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="I8" s="0" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="B9" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9" s="0">
-        <v>3</v>
-      </c>
-      <c r="D9" s="0">
-        <v>2126</v>
-      </c>
-      <c r="E9" s="0">
-        <v>2184</v>
-      </c>
-      <c r="F9" s="0">
-        <v>2585</v>
-      </c>
-      <c r="G9" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="H9" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="I9" s="0" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="C10" s="0">
-        <v>4</v>
-      </c>
-      <c r="D10" s="0">
-        <v>1929</v>
-      </c>
-      <c r="E10" s="0">
-        <v>1982</v>
-      </c>
-      <c r="F10" s="0">
-        <v>2383</v>
-      </c>
-      <c r="G10" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="H10" s="0" t="s">
-        <v>27</v>
-      </c>
-      <c r="I10" s="0" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11" s="0">
-        <v>5</v>
-      </c>
-      <c r="D11" s="0">
-        <v>1515</v>
-      </c>
-      <c r="E11" s="0">
-        <v>1551</v>
-      </c>
-      <c r="F11" s="0">
-        <v>1952</v>
-      </c>
-      <c r="G11" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="H11" s="0" t="s">
-        <v>28</v>
-      </c>
-      <c r="I11" s="0" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>